<commit_message>
chore: clean and update listings Excel template with 5 complete sample listings and images
</commit_message>
<xml_diff>
--- a/listings_template.xlsx
+++ b/listings_template.xlsx
@@ -397,17 +397,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I6"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="42.83203125" customWidth="1"/>
-    <col min="4" max="4" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="38.83203125" customWidth="1"/>
     <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
     <col min="7" max="7" width="14.83203125" customWidth="1"/>
-    <col min="8" max="8" width="50.83203125" customWidth="1"/>
-    <col min="9" max="9" width="45.83203125" customWidth="1"/>
+    <col min="8" max="8" width="75.83203125" customWidth="1"/>
+    <col min="9" max="9" width="60.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,25 +447,25 @@
         <v>Transport</v>
       </c>
       <c r="C2" t="str">
-        <v>City Express Low-Floor AC Bus Branding</v>
+        <v>Mumbai Western Line EMU Full Train Wrap</v>
       </c>
       <c r="D2" t="str">
-        <v>Delhi NCR</v>
+        <v>Mumbai (Churchgate to Virar)</v>
       </c>
       <c r="E2">
-        <v>45000</v>
+        <v>165000</v>
       </c>
       <c r="F2" t="str">
-        <v>Bus</v>
+        <v>Train</v>
       </c>
       <c r="G2">
-        <v>650000</v>
+        <v>1450000</v>
       </c>
       <c r="H2" t="str">
-        <v>High-frequency commuter bus wrapping covering prime arterial routes.</v>
+        <v>High-impact commuter wrap across 12-car local train network operating 18 hours daily across prime commercial corridors.</v>
       </c>
       <c r="I2" t="str">
-        <v>https://images.unsplash.com/photo-1570125909232-eb263c188f7e?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
+        <v>https://images.unsplash.com/photo-1565019011521-b0575cbb57c8?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
       </c>
     </row>
     <row r="3">
@@ -473,178 +473,120 @@
         <v>Transit</v>
       </c>
       <c r="B3" t="str">
-        <v>Transport</v>
+        <v>Bus Fleet</v>
       </c>
       <c r="C3" t="str">
-        <v>Delhi Metro Blue Line Full Train Wrap</v>
+        <v>Delhi DTC Electric Low-Floor Bus Full Wrap</v>
       </c>
       <c r="D3" t="str">
-        <v>Delhi / NCR</v>
+        <v>Delhi NCR (Ring Road &amp; Connaught Place)</v>
       </c>
       <c r="E3">
-        <v>185000</v>
+        <v>48000</v>
       </c>
       <c r="F3" t="str">
-        <v>Metro</v>
+        <v>Bus</v>
       </c>
       <c r="G3">
-        <v>1200000</v>
+        <v>680000</v>
       </c>
       <c r="H3" t="str">
-        <v>Full exterior wrap across 6-coach train traversing Dwarka to Noida/Vaishali.</v>
+        <v>Complete exterior vinyl wrap on air-conditioned electric buses covering high-dwell central Delhi routes.</v>
       </c>
       <c r="I3" t="str">
-        <v>https://images.unsplash.com/photo-1474487548417-781cb71495f3?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
+        <v>https://images.unsplash.com/photo-1570125909232-eb263c188f7e?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Transit</v>
+        <v>Outdoor</v>
       </c>
       <c r="B4" t="str">
-        <v>Transport</v>
+        <v>Billboards &amp; Unipoles</v>
       </c>
       <c r="C4" t="str">
-        <v>Suburban Express Electric Train Panel</v>
+        <v>Gurugram Cyber City Highway Mega Unipole</v>
       </c>
       <c r="D4" t="str">
-        <v>Mumbai</v>
+        <v>Gurugram (NH-48 Corridor)</v>
       </c>
       <c r="E4">
-        <v>95000</v>
+        <v>135000</v>
       </c>
       <c r="F4" t="str">
-        <v>Train</v>
+        <v>Billboard</v>
       </c>
       <c r="G4">
-        <v>900000</v>
+        <v>1100000</v>
       </c>
       <c r="H4" t="str">
-        <v>Internal commuter panel advertising across western railway network.</v>
+        <v>Front-lit iconic 60x30 ft arterial highway unipole facing non-stop corporate executive vehicular traffic.</v>
       </c>
       <c r="I4" t="str">
-        <v>https://images.unsplash.com/photo-1565019011521-b0575cbb57c8?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
+        <v>https://images.unsplash.com/photo-1449824913935-59a10b8d2000?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Transit</v>
+        <v>Outdoor</v>
       </c>
       <c r="B5" t="str">
-        <v>Metro Networks</v>
+        <v>Digital Hoardings</v>
       </c>
       <c r="C5" t="str">
-        <v>Metro Station Platform Screen Doors (PSD)</v>
+        <v>Bandra Reclamation Iconic Curved DOOH LED</v>
       </c>
       <c r="D5" t="str">
-        <v>Bengaluru (Namma Metro)</v>
+        <v>Mumbai (Western Express Highway)</v>
       </c>
       <c r="E5">
-        <v>75000</v>
+        <v>220000</v>
       </c>
       <c r="F5" t="str">
-        <v>Metro</v>
+        <v>Digital Screen</v>
       </c>
       <c r="G5">
-        <v>550000</v>
+        <v>1750000</v>
       </c>
       <c r="H5" t="str">
-        <v>Illuminated platform screen door branding at high-traffic interchange stations.</v>
+        <v>P6 high-brightness curved digital screen with dynamic day/night creative scheduling and motion video support.</v>
       </c>
       <c r="I5" t="str">
-        <v>https://images.unsplash.com/photo-1514565131-fce0801e5785?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
+        <v>https://images.unsplash.com/photo-1534430480872-3498386e7856?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Outdoor</v>
+        <v>Airport</v>
       </c>
       <c r="B6" t="str">
-        <v>Billboards &amp; Unipoles</v>
+        <v>Terminal Displays</v>
       </c>
       <c r="C6" t="str">
-        <v>Cyber City Arterial Unipole (Backlit)</v>
+        <v>IGI Terminal 3 Departure Security Concourse Totem</v>
       </c>
       <c r="D6" t="str">
-        <v>Gurugram</v>
+        <v>New Delhi Airport (T3 International)</v>
       </c>
       <c r="E6">
-        <v>125000</v>
+        <v>285000</v>
       </c>
       <c r="F6" t="str">
-        <v>Billboard</v>
+        <v>Digital Totem</v>
       </c>
       <c r="G6">
-        <v>980000</v>
+        <v>920000</v>
       </c>
       <c r="H6" t="str">
-        <v>Front-facing highway unipole catching top corporate commuters.</v>
+        <v>Ultra-HD 85-inch digital freestanding totem network positioned directly before international departures security gates.</v>
       </c>
       <c r="I6" t="str">
-        <v>https://images.unsplash.com/photo-1449824913935-59a10b8d2000?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Outdoor</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Digital Hoardings</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Bandra Flyover Curved DOOH Screen</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Mumbai</v>
-      </c>
-      <c r="E7">
-        <v>210000</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Digital Screen</v>
-      </c>
-      <c r="G7">
-        <v>1400000</v>
-      </c>
-      <c r="H7" t="str">
-        <v>P6 LED high-definition screen at Western Express Highway intersection.</v>
-      </c>
-      <c r="I7" t="str">
-        <v>https://images.unsplash.com/photo-1534430480872-3498386e7856?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>Airport</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Terminal Displays</v>
-      </c>
-      <c r="C8" t="str">
-        <v>T3 Departure Lounge Digital Totem</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Delhi Airport</v>
-      </c>
-      <c r="E8">
-        <v>275000</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Digital Totem</v>
-      </c>
-      <c r="G8">
-        <v>850000</v>
-      </c>
-      <c r="H8" t="str">
-        <v>Premium UHD digital totems targeting high-net-worth business travelers.</v>
-      </c>
-      <c r="I8" t="str">
         <v>https://images.unsplash.com/photo-1436491865332-7a61a109cc05?q=80&amp;w=800&amp;auto=format&amp;fit=crop</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>